<commit_message>
Inclui Responsável de Setor na ordem e Missão no modelo Excel
</commit_message>
<xml_diff>
--- a/modelo_planilha.xlsx
+++ b/modelo_planilha.xlsx
@@ -1,127 +1,88 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/douglasvital/Documents/Igreja/GeradorCrachas/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4534A7E-CFEB-A04A-88BC-654956F4A83C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="4340" yWindow="920" windowWidth="24460" windowHeight="15760" xr2:uid="{07CB6392-0428-F142-8680-68B070C8C622}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planilha1" sheetId="1" r:id="Rb315f2c4e7384dd9"/>
+  </x:sheets>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>Unidade</t>
-  </si>
-  <si>
-    <t>Nome Completo</t>
-  </si>
-  <si>
-    <t>Poltrona</t>
-  </si>
-  <si>
-    <t>Possuí Plano de Saúde?</t>
-  </si>
-  <si>
-    <t>Nome do Plano</t>
-  </si>
-  <si>
-    <t>Telefone do Plano</t>
-  </si>
-  <si>
-    <t>Nome Contato de Emergência</t>
-  </si>
-  <si>
-    <t>Telefone Contato de Emergência</t>
-  </si>
-  <si>
-    <t>Tipo de Contato</t>
-  </si>
-</sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:si>
+    <x:t xml:space="preserve">Unidade</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Nome Completo</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Poltrona</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Possuí Plano de Saúde?</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Nome do Plano</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Telefone do Plano</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Nome Contato de Emergência</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Telefone Contato de Emergência</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Tipo de Contato</x:t>
+  </x:si>
+</x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="3">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
-</styleSheet>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:fonts count="1">
+    <x:font>
+      <x:sz val="12"/>
+      <x:color theme="1"/>
+      <x:name val="Aptos Narrow"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="3">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor theme="0" tint="-0.15"/>
+      </x:patternFill>
+    </x:fill>
+  </x:fills>
+  <x:borders count="1">
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </x:cellStyleXfs>
+  <x:cellXfs count="2">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0"/>
+  </x:cellStyles>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -167,7 +128,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -219,7 +180,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -280,23 +241,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -306,23 +267,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -330,26 +291,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -384,17 +342,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -430,59 +388,56 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A12B043-080C-254D-9E9C-33B827194DCA}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <x:cols>
+    <x:col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <x:col min="4" max="4" width="20.1640625" customWidth="1"/>
+    <x:col min="5" max="5" width="13.1640625" customWidth="1"/>
+    <x:col min="6" max="6" width="15.1640625" customWidth="1"/>
+    <x:col min="7" max="7" width="25.33203125" customWidth="1"/>
+    <x:col min="8" max="8" width="27.5" customWidth="1"/>
+    <x:col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I1" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J1" s="1" t="str">
+        <x:v>Missão</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>